<commit_message>
feat : 나선수리검, 나선환, Behavior Tree
</commit_message>
<xml_diff>
--- a/Client/Bin/Resources/Data/xlsx/DT_SkilLData.xlsx
+++ b/Client/Bin/Resources/Data/xlsx/DT_SkilLData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitDesktop\Dx11_Naruto\Client\Bin\Resources\Data\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0F5E47C-6871-4072-8D07-AC2AB56C29CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{080176A6-0F61-4043-82CA-946B8A6E3F93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6FF045EB-CA47-4F87-A666-41B179691649}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>SkillID</t>
   </si>
@@ -34,10 +34,6 @@
     <t>Rasengan</t>
   </si>
   <si>
-    <t>Fireball</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>Chidori</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -67,6 +63,56 @@
   </si>
   <si>
     <t>Skill_RasenShuriken</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>BlastboomDance</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Skill_Chidori</t>
+  </si>
+  <si>
+    <t>Skill_BlastBoomDance</t>
+  </si>
+  <si>
+    <t>hasDashPhase</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>dashSpeed</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>maxDashDistance</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>targetStopDistance</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>attackEndAnimStateName</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Skill_Rasengan_End</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>airAnimStateName</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>airGravityOff</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Skill_Rasengan_Air</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Skill_RasenShuriken_Air</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1019,18 +1065,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7395922-27B8-4533-BFE6-6C196B1AE7C3}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="43.375" customWidth="1"/>
-    <col min="3" max="3" width="17.125" customWidth="1"/>
+    <col min="1" max="1" width="6.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="19.25" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="27.625" customWidth="1"/>
+    <col min="5" max="5" width="16.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.5" customWidth="1"/>
+    <col min="13" max="13" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1041,16 +1094,37 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
         <v>10</v>
       </c>
-      <c r="F1" t="s">
-        <v>11</v>
+      <c r="G1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1001</v>
       </c>
@@ -1061,27 +1135,48 @@
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E2">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>14</v>
+      </c>
+      <c r="I2">
+        <v>8</v>
+      </c>
+      <c r="J2">
+        <v>1.5</v>
+      </c>
+      <c r="K2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1002</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3">
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1089,8 +1184,26 @@
       <c r="F3" t="b">
         <v>0</v>
       </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>5</v>
+      </c>
+      <c r="I3">
+        <v>20</v>
+      </c>
+      <c r="J3">
+        <v>1.5</v>
+      </c>
+      <c r="L3" t="s">
+        <v>24</v>
+      </c>
+      <c r="M3" t="b">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1003</v>
       </c>
@@ -1100,36 +1213,72 @@
       <c r="C4">
         <v>5</v>
       </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
       <c r="E4">
+        <v>4</v>
+      </c>
+      <c r="F4" t="b">
         <v>1</v>
       </c>
-      <c r="F4" t="b">
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>5</v>
+      </c>
+      <c r="I4">
+        <v>20</v>
+      </c>
+      <c r="J4">
+        <v>1.5</v>
+      </c>
+      <c r="M4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1004</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
       <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>5</v>
+      </c>
+      <c r="I5">
+        <v>20</v>
+      </c>
+      <c r="J5">
+        <v>1.5</v>
+      </c>
+      <c r="M5" t="b">
         <v>1</v>
       </c>
-      <c r="F5" t="b">
-        <v>1</v>
-      </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1005</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C6">
         <v>5</v>
@@ -1139,6 +1288,21 @@
       </c>
       <c r="F6" t="b">
         <v>0</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>20</v>
+      </c>
+      <c r="J6">
+        <v>1.5</v>
+      </c>
+      <c r="M6" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>